<commit_message>
Tambah naskah lengkap konten IG minggu 1 (Siap TKA, Siap Mental)
Naskah carousel, Reels, dan infografis checklist untuk 19-23 Okt 2026,
lengkap dengan caption, alt text, catatan fasilitator, rencana Stories,
dan checklist produksi. Judul minggu 1 di kalender disesuaikan dengan
jadwal TKA nasional (26 Okt-8 Nov 2026).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018WWHGzf43cnjJy346VsAtj
</commit_message>
<xml_diff>
--- a/BK-Cigalontang/konten-instagram/kalender/Kalender_Konten_IG_BK_2026-2027.xlsx
+++ b/BK-Cigalontang/konten-instagram/kalender/Kalender_Konten_IG_BK_2026-2027.xlsx
@@ -696,7 +696,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Menjelang Prakiraan TKA (26–30 Okt); Bulan Kesehatan Mental</t>
+          <t>Menjelang TKA (nasional 26 Okt–8 Nov; sekolah: 26–30 Okt &amp; XII 2–6 Nov); Bulan Kesehatan Mental</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
@@ -768,7 +768,7 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Menjelang Prakiraan TKA (26–30 Okt); Bulan Kesehatan Mental</t>
+          <t>Menjelang TKA (nasional 26 Okt–8 Nov; sekolah: 26–30 Okt &amp; XII 2–6 Nov); Bulan Kesehatan Mental</t>
         </is>
       </c>
       <c r="I6" s="9" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="K6" s="8" t="inlineStr">
         <is>
-          <t>POV: H-7 TKA tapi Otak Nge-freeze</t>
+          <t>POV: H-5 TKA tapi Otak Nge-freeze</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Menjelang Prakiraan TKA (26–30 Okt); Bulan Kesehatan Mental</t>
+          <t>Menjelang TKA (nasional 26 Okt–8 Nov; sekolah: 26–30 Okt &amp; XII 2–6 Nov); Bulan Kesehatan Mental</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr">
@@ -850,12 +850,12 @@
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Single Image</t>
+          <t>Infografis</t>
         </is>
       </c>
       <c r="K7" s="8" t="inlineStr">
         <is>
-          <t>Checklist H-1 TKA</t>
+          <t>Checklist Sebelum TKA — Simpan untuk Hari-H</t>
         </is>
       </c>
       <c r="L7" s="5" t="inlineStr">
@@ -8547,7 +8547,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Menjelang Prakiraan TKA (26–30 Okt); Bulan Kesehatan Mental</t>
+          <t>Menjelang TKA (nasional 26 Okt–8 Nov; sekolah: 26–30 Okt &amp; XII 2–6 Nov); Bulan Kesehatan Mental</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
@@ -8557,12 +8557,12 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>[Reels] POV: H-7 TKA tapi Otak Nge-freeze</t>
+          <t>[Reels] POV: H-5 TKA tapi Otak Nge-freeze</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>[Single Image] Checklist H-1 TKA</t>
+          <t>[Infografis] Checklist Sebelum TKA — Simpan untuk Hari-H</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">

</xml_diff>